<commit_message>
data: hourly update 2026-06-28 14:52Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-06-28.xlsx
+++ b/data/output/workbook/2026-06-28.xlsx
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-28 08:19</t>
+          <t>2026-06-28 10:51</t>
         </is>
       </c>
     </row>
@@ -7972,7 +7972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8097,32 +8097,32 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
+          <t>Cincinnati Reds @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 163.5</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5769059405940594</v>
+        <v>0.6281900900900901</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-136</v>
+        <v>-169</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-102</v>
+        <v>-122</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 62.8% (fair -169). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -8158,17 +8158,17 @@
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Pittsburgh Pirates</t>
+          <t>Miami Marlins @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -8178,17 +8178,17 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.628525</v>
+        <v>0.4701680672268908</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-169</v>
+        <v>113</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-124</v>
+        <v>138</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -8212,7 +8212,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 62.9% (fair -169). Your call.</t>
+          <t>Model 47.0% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -8229,12 +8229,12 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -8244,17 +8244,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 166.5</t>
+          <t>Over 164.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5774549019607843</v>
+        <v>0.5506435643564357</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-137</v>
+        <v>-123</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-104</v>
+        <v>102</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -137). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -8290,17 +8290,17 @@
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
+          <t>Cincinnati Reds @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -8310,17 +8310,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Golden State Valkyries</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5862737089201878</v>
+        <v>0.6436134453781512</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-142</v>
+        <v>-181</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-113</v>
+        <v>-138</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 58.6% (fair -142). Your call.</t>
+          <t>Model 64.4% (fair -181). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -8361,32 +8361,32 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Las Vegas Aces @ Chicago Sky</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Golden State Valkyries</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.526298076923077</v>
+        <v>0.5885549295774647</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-111</v>
+        <v>-143</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>108</v>
+        <v>-113</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -8410,7 +8410,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 58.9% (fair -143). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -8427,32 +8427,32 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs @ Milwaukee Brewers</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.3882014388489208</v>
+        <v>0.5511731707317074</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>158</v>
+        <v>-123</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>178</v>
+        <v>-105</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -8476,7 +8476,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 38.8% (fair +158). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -8488,17 +8488,17 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Colorado Rockies</t>
+          <t>Texas Rangers @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -8508,17 +8508,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.473920704845815</v>
+        <v>0.4842342342342343</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -8559,12 +8559,12 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Milwaukee Brewers</t>
+          <t>Minnesota Twins @ Houston Astros</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -8574,17 +8574,17 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.6447000000000001</v>
+        <v>0.4944700460829493</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-181</v>
+        <v>102</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-150</v>
+        <v>117</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -8608,7 +8608,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 64.5% (fair -181). Your call.</t>
+          <t>Model 49.4% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -8620,17 +8620,17 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Houston Astros</t>
+          <t>Colorado Rockies @ Minnesota Twins</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -8640,17 +8640,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4944700460829493</v>
+        <v>0.4286</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>102</v>
+        <v>133</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>117</v>
+        <v>150</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 49.4% (fair +102). Your call.</t>
+          <t>Model 42.9% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -8691,12 +8691,12 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Toronto Blue Jays</t>
+          <t>Seattle Mariners @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -8706,17 +8706,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4873853211009175</v>
+        <v>0.53255</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>105</v>
+        <v>-114</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -8740,7 +8740,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 48.7% (fair +105). Your call.</t>
+          <t>Model 53.3% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -8757,12 +8757,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Baltimore Orioles</t>
+          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>22:35</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -8772,17 +8772,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4677533039647577</v>
+        <v>0.53215</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>114</v>
+        <v>-114</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -8806,7 +8806,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 46.8% (fair +114). Your call.</t>
+          <t>Model 53.2% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -8818,17 +8818,17 @@
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Seattle Mariners @ Cleveland Guardians</t>
+          <t>Detroit Tigers @ New York Yankees</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -8838,17 +8838,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.52885</v>
+        <v>0.4620264317180616</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-112</v>
+        <v>116</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -8872,7 +8872,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 46.2% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -8889,12 +8889,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Colorado Rockies @ Minnesota Twins</t>
+          <t>Arizona Diamondbacks @ Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -8904,17 +8904,17 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4366806722689076</v>
+        <v>0.3857777777777778</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>129</v>
+        <v>159</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>138</v>
+        <v>170</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 43.7% (fair +129). Your call.</t>
+          <t>Model 38.6% (fair +159). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -8950,17 +8950,17 @@
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks @ Tampa Bay Rays</t>
+          <t>Texas Rangers @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -8970,17 +8970,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.3847777777777777</v>
+        <v>0.4994711538461538</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>170</v>
+        <v>108</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -9004,7 +9004,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 38.5% (fair +160). Your call.</t>
+          <t>Model 49.9% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9016,37 +9016,37 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks @ Tampa Bay Rays</t>
+          <t>New York Mets @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>23:07</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5390653846153846</v>
+        <v>0.4985096153846154</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-117</v>
+        <v>101</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-108</v>
+        <v>108</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9070,7 +9070,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 49.9% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9087,12 +9087,12 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>New York Mets @ Toronto Blue Jays</t>
+          <t>Chicago White Sox @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>23:07</t>
+          <t>22:35</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -9102,17 +9102,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4985096153846154</v>
+        <v>0.4563876651982379</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9136,7 +9136,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 49.9% (fair +101). Your call.</t>
+          <t>Model 45.6% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9148,17 +9148,17 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Cleveland Guardians</t>
+          <t>Chicago Cubs @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -9168,17 +9168,17 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4967788461538462</v>
+        <v>0.4045703125</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>101</v>
+        <v>147</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>108</v>
+        <v>156</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 40.5% (fair +147). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9219,12 +9219,12 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Las Vegas Aces @ Chicago Sky</t>
+          <t>Houston Astros @ Detroit Tigers</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
@@ -9234,17 +9234,17 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Las Vegas Aces</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.733295652173913</v>
+        <v>0.4763594470046084</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-275</v>
+        <v>110</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-245</v>
+        <v>117</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 73.3% (fair -275). Your call.</t>
+          <t>Model 47.6% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -9285,32 +9285,32 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Houston Astros @ Detroit Tigers</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Portland Fire +6.5</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4708675799086758</v>
+        <v>0.5117326732673267</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>112</v>
+        <v>-105</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 47.1% (fair +112). Your call.</t>
+          <t>Model 51.2% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -9370,13 +9370,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5768709251101322</v>
+        <v>0.5759203539823009</v>
       </c>
       <c r="G24" s="14" t="n">
         <v>-136</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-127</v>
+        <v>-126</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 57.6% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -9436,13 +9436,13 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.6238171875</v>
+        <v>0.6202444444444444</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-166</v>
+        <v>-163</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-156</v>
+        <v>-152</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 62.4% (fair -166). Your call.</t>
+          <t>Model 62.0% (fair -163). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -9475,9 +9475,141 @@
         <v/>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Las Vegas Aces @ Chicago Sky</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>Las Vegas Aces</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.7361574229691876</v>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>-279</v>
+      </c>
+      <c r="H26" s="15" t="n">
+        <v>-257</v>
+      </c>
+      <c r="I26" s="13">
+        <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
+        <v/>
+      </c>
+      <c r="J26" s="16">
+        <f>IF($H$26="","",$F$26*IF($H$26&lt;0,-100/$H$26,$H$26/100)-(1-$F$26))</f>
+        <v/>
+      </c>
+      <c r="K26" s="17">
+        <f>IF($H$26="","",MAX(0,($F$26*IF($H$26&lt;0,-100/$H$26,$H$26/100)-(1-$F$26))/IF($H$26&lt;0,-100/$H$26,$H$26/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L26" s="18">
+        <f>IF($H$26="","",ROUND(MIN($K$26,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M26" s="12">
+        <f>IF($J$26="","",IF($J$26&lt;0,"Pass",IF($J$26&lt;'Settings'!$B$4,"Thin",IF($J$26&lt;0.06,"✅ Sharp band",IF($J$26&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N26" s="19" t="inlineStr">
+        <is>
+          <t>Model 73.6% (fair -279). Your call.</t>
+        </is>
+      </c>
+      <c r="O26" s="15" t="n"/>
+      <c r="P26" s="16">
+        <f>IF(OR($H$26="",$O$26=""),"",(1+IF($H$26&lt;0,-100/$H$26,$H$26/100))/(1+IF($O$26&lt;0,-100/$O$26,$O$26/100))-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Washington Nationals @ Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="n">
+        <v>0.6464544117647059</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>-183</v>
+      </c>
+      <c r="H27" s="15" t="n">
+        <v>-172</v>
+      </c>
+      <c r="I27" s="13">
+        <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
+        <v/>
+      </c>
+      <c r="J27" s="16">
+        <f>IF($H$27="","",$F$27*IF($H$27&lt;0,-100/$H$27,$H$27/100)-(1-$F$27))</f>
+        <v/>
+      </c>
+      <c r="K27" s="17">
+        <f>IF($H$27="","",MAX(0,($F$27*IF($H$27&lt;0,-100/$H$27,$H$27/100)-(1-$F$27))/IF($H$27&lt;0,-100/$H$27,$H$27/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L27" s="18">
+        <f>IF($H$27="","",ROUND(MIN($K$27,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M27" s="12">
+        <f>IF($J$27="","",IF($J$27&lt;0,"Pass",IF($J$27&lt;'Settings'!$B$4,"Thin",IF($J$27&lt;0.06,"✅ Sharp band",IF($J$27&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N27" s="19" t="inlineStr">
+        <is>
+          <t>Model 64.6% (fair -183). Your call.</t>
+        </is>
+      </c>
+      <c r="O27" s="15" t="n"/>
+      <c r="P27" s="16">
+        <f>IF(OR($H$27="",$O$27=""),"",(1+IF($H$27&lt;0,-100/$H$27,$H$27/100))/(1+IF($O$27&lt;0,-100/$O$27,$O$27/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J25">
+  <conditionalFormatting sqref="J5:J27">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -9643,13 +9775,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.3512132352941177</v>
+        <v>0.3535185185185185</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -9673,7 +9805,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 35.1% (fair +185). Your call.</t>
+          <t>Model 35.4% (fair +183). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -9709,13 +9841,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6488035971223022</v>
+        <v>0.6464544117647059</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-185</v>
+        <v>-183</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-178</v>
+        <v>-172</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -9739,7 +9871,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 64.9% (fair -185). Your call.</t>
+          <t>Model 64.6% (fair -183). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -9781,7 +9913,7 @@
         <v>-136</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -9913,7 +10045,7 @@
         <v>-116</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -9979,7 +10111,7 @@
         <v>116</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -10039,13 +10171,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.3714864864864865</v>
+        <v>0.3718385650224215</v>
       </c>
       <c r="G11" s="14" t="n">
         <v>169</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -10069,7 +10201,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 37.1% (fair +169). Your call.</t>
+          <t>Model 37.2% (fair +169). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -10105,13 +10237,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.628525</v>
+        <v>0.6281900900900901</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>-169</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-124</v>
+        <v>-122</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -10135,7 +10267,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 62.9% (fair -169). Your call.</t>
+          <t>Model 62.8% (fair -169). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -10167,7 +10299,7 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
@@ -10177,7 +10309,7 @@
         <v>-116</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -10233,7 +10365,7 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
@@ -10243,7 +10375,7 @@
         <v>116</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -10375,7 +10507,7 @@
         <v>136</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-122</v>
+        <v>-123</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -10435,13 +10567,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4873853211009175</v>
+        <v>0.4842342342342343</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -10465,7 +10597,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 48.7% (fair +105). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -10501,13 +10633,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5126181818181818</v>
+        <v>0.5157522522522523</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-105</v>
+        <v>-107</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-120</v>
+        <v>-122</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -10531,7 +10663,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 51.3% (fair -105). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -10573,7 +10705,7 @@
         <v>-126</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>100</v>
+        <v>-102</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -10639,7 +10771,7 @@
         <v>126</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -10831,13 +10963,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5291612612612613</v>
+        <v>0.5236197183098591</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-112</v>
+        <v>-110</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>-122</v>
+        <v>-113</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -10861,7 +10993,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 52.4% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -10897,13 +11029,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.4708675799086758</v>
+        <v>0.4763594470046084</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -10927,7 +11059,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 47.1% (fair +112). Your call.</t>
+          <t>Model 47.6% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -11035,7 +11167,7 @@
         <v>123</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -11095,10 +11227,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.52885</v>
+        <v>0.53255</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-112</v>
+        <v>-114</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>100</v>
@@ -11125,7 +11257,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 53.3% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -11161,13 +11293,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4711098039215686</v>
+        <v>0.4674752475247525</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-104</v>
+        <v>102</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -11191,7 +11323,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 47.1% (fair +112). Your call.</t>
+          <t>Model 46.7% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -11233,7 +11365,7 @@
         <v>176</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -11299,7 +11431,7 @@
         <v>-176</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -11431,7 +11563,7 @@
         <v>-244</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -11491,10 +11623,10 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.3847777777777777</v>
+        <v>0.3857777777777778</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H33" s="15" t="n">
         <v>170</v>
@@ -11521,7 +11653,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 38.5% (fair +160). Your call.</t>
+          <t>Model 38.6% (fair +159). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -11557,13 +11689,13 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.6152233576642336</v>
+        <v>0.6142037037037037</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-160</v>
+        <v>-159</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>-174</v>
+        <v>-170</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -11587,7 +11719,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 61.5% (fair -160). Your call.</t>
+          <t>Model 61.4% (fair -159). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -11619,17 +11751,17 @@
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Over 8</t>
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.5390653846153846</v>
+        <v>0.4802</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>-117</v>
+        <v>108</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>-108</v>
+        <v>107</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -11653,7 +11785,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -11685,17 +11817,17 @@
       </c>
       <c r="E36" s="20" t="inlineStr">
         <is>
-          <t>Under 7.5</t>
+          <t>Under 8</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.4609223300970874</v>
+        <v>0.5198</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>117</v>
+        <v>-108</v>
       </c>
       <c r="H36" s="15" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I36" s="13">
         <f>IF($H$36="","",IF($H$36&lt;0,-$H$36/(-$H$36+100),100/($H$36+100)))</f>
@@ -11719,7 +11851,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 52.0% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -11755,10 +11887,10 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.4526</v>
+        <v>0.4498222222222222</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H37" s="15" t="n">
         <v>125</v>
@@ -11785,7 +11917,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 45.0% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -11821,13 +11953,13 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5474</v>
+        <v>0.5501540540540542</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>-121</v>
+        <v>-122</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>120</v>
+        <v>-122</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -11851,7 +11983,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -11887,13 +12019,13 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.5764094420600858</v>
+        <v>0.5788462184873949</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>-136</v>
+        <v>-137</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>-133</v>
+        <v>-138</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -11917,7 +12049,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 57.6% (fair -136). Your call.</t>
+          <t>Model 57.9% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -11953,13 +12085,13 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.4236051502145923</v>
+        <v>0.4211538461538462</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -11983,7 +12115,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 42.4% (fair +136). Your call.</t>
+          <t>Model 42.1% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -12025,7 +12157,7 @@
         <v>136</v>
       </c>
       <c r="H41" s="15" t="n">
-        <v>117</v>
+        <v>104</v>
       </c>
       <c r="I41" s="13">
         <f>IF($H$41="","",IF($H$41&lt;0,-$H$41/(-$H$41+100),100/($H$41+100)))</f>
@@ -12091,7 +12223,7 @@
         <v>-136</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="I42" s="13">
         <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
@@ -12151,13 +12283,13 @@
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>0.4366806722689076</v>
+        <v>0.4286</v>
       </c>
       <c r="G43" s="14" t="n">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="I43" s="13">
         <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
@@ -12181,7 +12313,7 @@
       </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>Model 43.7% (fair +129). Your call.</t>
+          <t>Model 42.9% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O43" s="15" t="n"/>
@@ -12217,13 +12349,13 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.5633067226890757</v>
+        <v>0.5713967213114753</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>-129</v>
+        <v>-133</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>-138</v>
+        <v>-144</v>
       </c>
       <c r="I44" s="13">
         <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
@@ -12247,7 +12379,7 @@
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 57.1% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O44" s="15" t="n"/>
@@ -12289,7 +12421,7 @@
         <v>-110</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -12355,7 +12487,7 @@
         <v>110</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I46" s="13">
         <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
@@ -12421,7 +12553,7 @@
         <v>138</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I47" s="13">
         <f>IF($H$47="","",IF($H$47&lt;0,-$H$47/(-$H$47+100),100/($H$47+100)))</f>
@@ -12487,7 +12619,7 @@
         <v>-138</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>-107</v>
+        <v>101</v>
       </c>
       <c r="I48" s="13">
         <f>IF($H$48="","",IF($H$48&lt;0,-$H$48/(-$H$48+100),100/($H$48+100)))</f>
@@ -12547,13 +12679,13 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>0.4231111111111111</v>
+        <v>0.4241071428571428</v>
       </c>
       <c r="G49" s="14" t="n">
         <v>136</v>
       </c>
       <c r="H49" s="15" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I49" s="13">
         <f>IF($H$49="","",IF($H$49&lt;0,-$H$49/(-$H$49+100),100/($H$49+100)))</f>
@@ -12577,7 +12709,7 @@
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 42.4% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O49" s="15" t="n"/>
@@ -12613,13 +12745,13 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.5768709251101322</v>
+        <v>0.5759203539823009</v>
       </c>
       <c r="G50" s="14" t="n">
         <v>-136</v>
       </c>
       <c r="H50" s="15" t="n">
-        <v>-127</v>
+        <v>-126</v>
       </c>
       <c r="I50" s="13">
         <f>IF($H$50="","",IF($H$50&lt;0,-$H$50/(-$H$50+100),100/($H$50+100)))</f>
@@ -12643,7 +12775,7 @@
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 57.6% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O50" s="15" t="n"/>
@@ -12685,7 +12817,7 @@
         <v>-131</v>
       </c>
       <c r="H51" s="15" t="n">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="I51" s="13">
         <f>IF($H$51="","",IF($H$51&lt;0,-$H$51/(-$H$51+100),100/($H$51+100)))</f>
@@ -12751,7 +12883,7 @@
         <v>131</v>
       </c>
       <c r="H52" s="15" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="I52" s="13">
         <f>IF($H$52="","",IF($H$52&lt;0,-$H$52/(-$H$52+100),100/($H$52+100)))</f>
@@ -12817,7 +12949,7 @@
         <v>112</v>
       </c>
       <c r="H53" s="15" t="n">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="I53" s="13">
         <f>IF($H$53="","",IF($H$53&lt;0,-$H$53/(-$H$53+100),100/($H$53+100)))</f>
@@ -12943,13 +13075,13 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.3882014388489208</v>
+        <v>0.4045703125</v>
       </c>
       <c r="G55" s="14" t="n">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="H55" s="15" t="n">
-        <v>178</v>
+        <v>156</v>
       </c>
       <c r="I55" s="13">
         <f>IF($H$55="","",IF($H$55&lt;0,-$H$55/(-$H$55+100),100/($H$55+100)))</f>
@@ -12973,7 +13105,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 38.8% (fair +158). Your call.</t>
+          <t>Model 40.5% (fair +147). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -13009,13 +13141,13 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.6118297872340425</v>
+        <v>0.5954203125</v>
       </c>
       <c r="G56" s="14" t="n">
-        <v>-158</v>
+        <v>-147</v>
       </c>
       <c r="H56" s="15" t="n">
-        <v>-182</v>
+        <v>-156</v>
       </c>
       <c r="I56" s="13">
         <f>IF($H$56="","",IF($H$56&lt;0,-$H$56/(-$H$56+100),100/($H$56+100)))</f>
@@ -13039,7 +13171,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 61.2% (fair -158). Your call.</t>
+          <t>Model 59.5% (fair -147). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -13081,7 +13213,7 @@
         <v>-146</v>
       </c>
       <c r="H57" s="15" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I57" s="13">
         <f>IF($H$57="","",IF($H$57&lt;0,-$H$57/(-$H$57+100),100/($H$57+100)))</f>
@@ -13147,7 +13279,7 @@
         <v>146</v>
       </c>
       <c r="H58" s="15" t="n">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="I58" s="13">
         <f>IF($H$58="","",IF($H$58&lt;0,-$H$58/(-$H$58+100),100/($H$58+100)))</f>
@@ -13207,13 +13339,13 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.4565437788018433</v>
+        <v>0.4523</v>
       </c>
       <c r="G59" s="14" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H59" s="15" t="n">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="I59" s="13">
         <f>IF($H$59="","",IF($H$59&lt;0,-$H$59/(-$H$59+100),100/($H$59+100)))</f>
@@ -13237,7 +13369,7 @@
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>Model 45.7% (fair +119). Your call.</t>
+          <t>Model 45.2% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O59" s="15" t="n"/>
@@ -13273,13 +13405,13 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.5434299539170507</v>
+        <v>0.5477000000000001</v>
       </c>
       <c r="G60" s="14" t="n">
-        <v>-119</v>
+        <v>-121</v>
       </c>
       <c r="H60" s="15" t="n">
-        <v>-117</v>
+        <v>104</v>
       </c>
       <c r="I60" s="13">
         <f>IF($H$60="","",IF($H$60&lt;0,-$H$60/(-$H$60+100),100/($H$60+100)))</f>
@@ -13303,7 +13435,7 @@
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 54.8% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O60" s="15" t="n"/>
@@ -13915,13 +14047,13 @@
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>0.4676061674008811</v>
+        <v>0.4675938053097345</v>
       </c>
       <c r="G70" s="14" t="n">
         <v>114</v>
       </c>
       <c r="H70" s="15" t="n">
-        <v>-127</v>
+        <v>-126</v>
       </c>
       <c r="I70" s="13">
         <f>IF($H$70="","",IF($H$70&lt;0,-$H$70/(-$H$70+100),100/($H$70+100)))</f>
@@ -13987,7 +14119,7 @@
         <v>134</v>
       </c>
       <c r="H71" s="15" t="n">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="I71" s="13">
         <f>IF($H$71="","",IF($H$71&lt;0,-$H$71/(-$H$71+100),100/($H$71+100)))</f>
@@ -14053,7 +14185,7 @@
         <v>-134</v>
       </c>
       <c r="H72" s="15" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="I72" s="13">
         <f>IF($H$72="","",IF($H$72&lt;0,-$H$72/(-$H$72+100),100/($H$72+100)))</f>
@@ -14113,13 +14245,13 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.33796875</v>
+        <v>0.3379615384615385</v>
       </c>
       <c r="G73" s="14" t="n">
         <v>196</v>
       </c>
       <c r="H73" s="15" t="n">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="I73" s="13">
         <f>IF($H$73="","",IF($H$73&lt;0,-$H$73/(-$H$73+100),100/($H$73+100)))</f>
@@ -14243,10 +14375,10 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>0.4677533039647577</v>
+        <v>0.4563876651982379</v>
       </c>
       <c r="G75" s="14" t="n">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="H75" s="15" t="n">
         <v>127</v>
@@ -14273,7 +14405,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Model 46.8% (fair +114). Your call.</t>
+          <t>Model 45.6% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O75" s="15" t="n"/>
@@ -14309,13 +14441,13 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.5322251101321587</v>
+        <v>0.5436504201680672</v>
       </c>
       <c r="G76" s="14" t="n">
-        <v>-114</v>
+        <v>-119</v>
       </c>
       <c r="H76" s="15" t="n">
-        <v>-127</v>
+        <v>-138</v>
       </c>
       <c r="I76" s="13">
         <f>IF($H$76="","",IF($H$76&lt;0,-$H$76/(-$H$76+100),100/($H$76+100)))</f>
@@ -14339,7 +14471,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Model 53.2% (fair -114). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O76" s="15" t="n"/>
@@ -14375,13 +14507,13 @@
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>0.5033803921568627</v>
+        <v>0.53215</v>
       </c>
       <c r="G77" s="14" t="n">
-        <v>-101</v>
+        <v>-114</v>
       </c>
       <c r="H77" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I77" s="13">
         <f>IF($H$77="","",IF($H$77&lt;0,-$H$77/(-$H$77+100),100/($H$77+100)))</f>
@@ -14405,7 +14537,7 @@
       </c>
       <c r="N77" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 53.2% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O77" s="15" t="n"/>
@@ -14441,10 +14573,10 @@
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.4966</v>
+        <v>0.46785</v>
       </c>
       <c r="G78" s="14" t="n">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="H78" s="15" t="n">
         <v>100</v>
@@ -14471,7 +14603,7 @@
       </c>
       <c r="N78" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 46.8% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O78" s="15" t="n"/>
@@ -14507,13 +14639,13 @@
         </is>
       </c>
       <c r="F79" s="13" t="n">
-        <v>0.4885</v>
+        <v>0.4620264317180616</v>
       </c>
       <c r="G79" s="14" t="n">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="H79" s="15" t="n">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="I79" s="13">
         <f>IF($H$79="","",IF($H$79&lt;0,-$H$79/(-$H$79+100),100/($H$79+100)))</f>
@@ -14537,7 +14669,7 @@
       </c>
       <c r="N79" s="19" t="inlineStr">
         <is>
-          <t>Model 48.9% (fair +105). Your call.</t>
+          <t>Model 46.2% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O79" s="15" t="n"/>
@@ -14573,13 +14705,13 @@
         </is>
       </c>
       <c r="F80" s="13" t="n">
-        <v>0.5115</v>
+        <v>0.5379364806866953</v>
       </c>
       <c r="G80" s="14" t="n">
-        <v>-105</v>
+        <v>-116</v>
       </c>
       <c r="H80" s="15" t="n">
-        <v>-127</v>
+        <v>-133</v>
       </c>
       <c r="I80" s="13">
         <f>IF($H$80="","",IF($H$80&lt;0,-$H$80/(-$H$80+100),100/($H$80+100)))</f>
@@ -14603,7 +14735,7 @@
       </c>
       <c r="N80" s="19" t="inlineStr">
         <is>
-          <t>Model 51.1% (fair -105). Your call.</t>
+          <t>Model 53.8% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O80" s="15" t="n"/>
@@ -14777,7 +14909,7 @@
         <v>-102</v>
       </c>
       <c r="H83" s="15" t="n">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="I83" s="13">
         <f>IF($H$83="","",IF($H$83&lt;0,-$H$83/(-$H$83+100),100/($H$83+100)))</f>
@@ -14903,10 +15035,10 @@
         </is>
       </c>
       <c r="F85" s="13" t="n">
-        <v>0.4967788461538462</v>
+        <v>0.4994711538461538</v>
       </c>
       <c r="G85" s="14" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H85" s="15" t="n">
         <v>108</v>
@@ -14933,7 +15065,7 @@
       </c>
       <c r="N85" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 49.9% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O85" s="15" t="n"/>
@@ -14969,13 +15101,13 @@
         </is>
       </c>
       <c r="F86" s="13" t="n">
-        <v>0.5031948356807512</v>
+        <v>0.5005384615384615</v>
       </c>
       <c r="G86" s="14" t="n">
-        <v>-101</v>
+        <v>-100</v>
       </c>
       <c r="H86" s="15" t="n">
-        <v>-113</v>
+        <v>-108</v>
       </c>
       <c r="I86" s="13">
         <f>IF($H$86="","",IF($H$86&lt;0,-$H$86/(-$H$86+100),100/($H$86+100)))</f>
@@ -14999,7 +15131,7 @@
       </c>
       <c r="N86" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O86" s="15" t="n"/>
@@ -15035,13 +15167,13 @@
         </is>
       </c>
       <c r="F87" s="13" t="n">
-        <v>0.3552941176470589</v>
+        <v>0.3563934426229509</v>
       </c>
       <c r="G87" s="14" t="n">
         <v>181</v>
       </c>
       <c r="H87" s="15" t="n">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="I87" s="13">
         <f>IF($H$87="","",IF($H$87&lt;0,-$H$87/(-$H$87+100),100/($H$87+100)))</f>
@@ -15065,7 +15197,7 @@
       </c>
       <c r="N87" s="19" t="inlineStr">
         <is>
-          <t>Model 35.5% (fair +181). Your call.</t>
+          <t>Model 35.6% (fair +181). Your call.</t>
         </is>
       </c>
       <c r="O87" s="15" t="n"/>
@@ -15101,13 +15233,13 @@
         </is>
       </c>
       <c r="F88" s="13" t="n">
-        <v>0.6447000000000001</v>
+        <v>0.6436134453781512</v>
       </c>
       <c r="G88" s="14" t="n">
         <v>-181</v>
       </c>
       <c r="H88" s="15" t="n">
-        <v>-150</v>
+        <v>-138</v>
       </c>
       <c r="I88" s="13">
         <f>IF($H$88="","",IF($H$88&lt;0,-$H$88/(-$H$88+100),100/($H$88+100)))</f>
@@ -15131,7 +15263,7 @@
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>Model 64.5% (fair -181). Your call.</t>
+          <t>Model 64.4% (fair -181). Your call.</t>
         </is>
       </c>
       <c r="O88" s="15" t="n"/>
@@ -15167,10 +15299,10 @@
         </is>
       </c>
       <c r="F89" s="13" t="n">
-        <v>0.4338325991189427</v>
+        <v>0.435726872246696</v>
       </c>
       <c r="G89" s="14" t="n">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H89" s="15" t="n">
         <v>127</v>
@@ -15197,7 +15329,7 @@
       </c>
       <c r="N89" s="19" t="inlineStr">
         <is>
-          <t>Model 43.4% (fair +131). Your call.</t>
+          <t>Model 43.6% (fair +130). Your call.</t>
         </is>
       </c>
       <c r="O89" s="15" t="n"/>
@@ -15233,13 +15365,13 @@
         </is>
       </c>
       <c r="F90" s="13" t="n">
-        <v>0.5662058823529411</v>
+        <v>0.5642510729613734</v>
       </c>
       <c r="G90" s="14" t="n">
-        <v>-131</v>
+        <v>-129</v>
       </c>
       <c r="H90" s="15" t="n">
-        <v>-138</v>
+        <v>-133</v>
       </c>
       <c r="I90" s="13">
         <f>IF($H$90="","",IF($H$90&lt;0,-$H$90/(-$H$90+100),100/($H$90+100)))</f>
@@ -15263,7 +15395,7 @@
       </c>
       <c r="N90" s="19" t="inlineStr">
         <is>
-          <t>Model 56.6% (fair -131). Your call.</t>
+          <t>Model 56.4% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O90" s="15" t="n"/>
@@ -15431,13 +15563,13 @@
         </is>
       </c>
       <c r="F93" s="13" t="n">
-        <v>0.5260800000000001</v>
+        <v>0.5297901639344262</v>
       </c>
       <c r="G93" s="14" t="n">
-        <v>-111</v>
+        <v>-113</v>
       </c>
       <c r="H93" s="15" t="n">
-        <v>-150</v>
+        <v>-144</v>
       </c>
       <c r="I93" s="13">
         <f>IF($H$93="","",IF($H$93&lt;0,-$H$93/(-$H$93+100),100/($H$93+100)))</f>
@@ -15461,7 +15593,7 @@
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 53.0% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O93" s="15" t="n"/>
@@ -15497,13 +15629,13 @@
         </is>
       </c>
       <c r="F94" s="13" t="n">
-        <v>0.473920704845815</v>
+        <v>0.4701680672268908</v>
       </c>
       <c r="G94" s="14" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H94" s="15" t="n">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="I94" s="13">
         <f>IF($H$94="","",IF($H$94&lt;0,-$H$94/(-$H$94+100),100/($H$94+100)))</f>
@@ -15527,7 +15659,7 @@
       </c>
       <c r="N94" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 47.0% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O94" s="15" t="n"/>
@@ -16088,13 +16220,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6238171875</v>
+        <v>0.6202444444444444</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-166</v>
+        <v>-163</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-156</v>
+        <v>-152</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -16118,7 +16250,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 62.4% (fair -166). Your call.</t>
+          <t>Model 62.0% (fair -163). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -16154,13 +16286,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.3761960784313726</v>
+        <v>0.37976</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -16184,7 +16316,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 37.6% (fair +166). Your call.</t>
+          <t>Model 38.0% (fair +163). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -16216,17 +16348,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Over 178.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.3591705069124424</v>
+        <v>0.3844</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -16250,7 +16382,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 35.9% (fair +178). Your call.</t>
+          <t>Model 38.4% (fair +160). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -16282,17 +16414,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 179.5</t>
+          <t>Under 178.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.6408</v>
+        <v>0.6155999999999999</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-178</v>
+        <v>-160</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -16316,7 +16448,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 64.1% (fair -178). Your call.</t>
+          <t>Model 61.6% (fair -160). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -16348,17 +16480,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Dallas Wings +3.5</t>
+          <t>Dallas Wings +2.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.4792</v>
+        <v>0.4447</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -16382,7 +16514,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 47.9% (fair +109). Your call.</t>
+          <t>Model 44.5% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -16414,14 +16546,14 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Lynx -3.5</t>
+          <t>Minnesota Lynx -2.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5207999999999999</v>
+        <v>0.5553</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-109</v>
+        <v>-125</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>113</v>
@@ -16448,7 +16580,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 52.1% (fair -109). Your call.</t>
+          <t>Model 55.5% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -16484,13 +16616,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.3053939393939394</v>
+        <v>0.3044444444444445</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -16514,7 +16646,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 30.5% (fair +227). Your call.</t>
+          <t>Model 30.4% (fair +228). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -16550,10 +16682,10 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.6945918918918919</v>
+        <v>0.6955714714714715</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-227</v>
+        <v>-228</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>-233</v>
@@ -16580,7 +16712,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 69.5% (fair -227). Your call.</t>
+          <t>Model 69.6% (fair -228). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -16612,17 +16744,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 166.5</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5774549019607843</v>
+        <v>0.5511731707317074</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-137</v>
+        <v>-123</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-104</v>
+        <v>-105</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -16646,7 +16778,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -137). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -16678,17 +16810,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 166.5</t>
+          <t>Under 167.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4226</v>
+        <v>0.4488</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-104</v>
+        <v>-105</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -16712,7 +16844,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +137). Your call.</t>
+          <t>Model 44.9% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -16744,17 +16876,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics -7.5</t>
+          <t>Washington Mystics -6.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4395</v>
+        <v>0.48825</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>128</v>
+        <v>105</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -16778,7 +16910,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 44.0% (fair +128). Your call.</t>
+          <t>Model 48.8% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -16810,17 +16942,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire +7.5</t>
+          <t>Portland Fire +6.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5605</v>
+        <v>0.5117326732673267</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-128</v>
+        <v>-105</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-104</v>
+        <v>102</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -16844,7 +16976,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 56.0% (fair -128). Your call.</t>
+          <t>Model 51.2% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -16880,13 +17012,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.733295652173913</v>
+        <v>0.7361574229691876</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-275</v>
+        <v>-279</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>-245</v>
+        <v>-257</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -16910,7 +17042,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 73.3% (fair -275). Your call.</t>
+          <t>Model 73.6% (fair -279). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -16946,13 +17078,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2638</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -16976,7 +17108,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 26.7% (fair +275). Your call.</t>
+          <t>Model 26.4% (fair +279). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -17008,14 +17140,14 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Over 181.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.526298076923077</v>
+        <v>0.4731730769230769</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-111</v>
+        <v>111</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>108</v>
@@ -17042,7 +17174,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 47.3% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -17074,14 +17206,14 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 179.5</t>
+          <t>Under 181.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4737</v>
+        <v>0.5267999999999999</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>111</v>
+        <v>-111</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>108</v>
@@ -17108,7 +17240,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 52.7% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -17140,17 +17272,17 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Chicago Sky -1.5</t>
+          <t>Chicago Sky +5.5</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.2046</v>
+        <v>0.4143</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>389</v>
+        <v>141</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -17174,7 +17306,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 20.5% (fair +389). Your call.</t>
+          <t>Model 41.4% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -17206,17 +17338,17 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Las Vegas Aces +1.5</t>
+          <t>Las Vegas Aces -5.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.7954</v>
+        <v>0.5857</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-389</v>
+        <v>-141</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -17240,7 +17372,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 79.5% (fair -389). Your call.</t>
+          <t>Model 58.6% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -17276,13 +17408,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4137558685446009</v>
+        <v>0.4114285714285715</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -17306,7 +17438,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 41.4% (fair +142). Your call.</t>
+          <t>Model 41.1% (fair +143). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -17342,10 +17474,10 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5862737089201878</v>
+        <v>0.5885549295774647</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-142</v>
+        <v>-143</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>-113</v>
@@ -17372,7 +17504,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 58.6% (fair -142). Your call.</t>
+          <t>Model 58.9% (fair -143). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -17404,17 +17536,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 163.5</t>
+          <t>Over 164.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5769059405940594</v>
+        <v>0.5506435643564357</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-136</v>
+        <v>-123</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-102</v>
+        <v>102</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -17438,7 +17570,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -17470,17 +17602,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 163.5</t>
+          <t>Under 164.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4231</v>
+        <v>0.4493</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-102</v>
+        <v>102</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -17504,7 +17636,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 44.9% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -17546,7 +17678,7 @@
         <v>-145</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -17612,7 +17744,7 @@
         <v>145</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>

</xml_diff>